<commit_message>
Update daily rolling forecast for 2026-08-24
</commit_message>
<xml_diff>
--- a/data/2026_08/snapshots/2026_08_24/dashboard_v3.xlsx
+++ b/data/2026_08/snapshots/2026_08_24/dashboard_v3.xlsx
@@ -491,13 +491,13 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>19759545</v>
+        <v>19762241</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>21805410</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-2045865</v>
+        <v>-2043169</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>-9.4</v>
@@ -515,13 +515,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>21717097</v>
+        <v>21719793</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>21805410</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-88313</v>
+        <v>-85617</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>-0.4</v>
@@ -539,13 +539,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>12736623</v>
+        <v>12739319</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>13393890</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>-657267</v>
+        <v>-654571</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>-4.9</v>
@@ -635,16 +635,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>1439</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>-52</v>
+        <v>-51</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-3.6</v>
+        <v>-3.5</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -707,16 +707,16 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>806</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>12</v>
+        <v>12.3</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>現時点着地見込み 1,976万円は前年同月 2,181万円を下回る見込み（前年差 ▲205万・-9.4%）。一方、通常営業ベース 2,172万円は前年を下回る（-0.4%）。差 ▲196万は通常営業ベースとの差であり、自費売上化と他曜日充足で埋められるかが焦点。</t>
+          <t>現時点着地見込み 1,976万円は前年同月 2,181万円を下回る見込み（前年差 ▲204万・-9.4%）。一方、通常営業ベース 2,172万円は前年を下回る（-0.4%）。差 ▲196万は通常営業ベースとの差であり、自費売上化と他曜日充足で埋められるかが焦点。</t>
         </is>
       </c>
     </row>

</xml_diff>